<commit_message>
view all the entered employee in the setting page of employee and enable edit department a section of them
</commit_message>
<xml_diff>
--- a/ClientApp/employeeTable.xlsx
+++ b/ClientApp/employeeTable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haya\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haya\source\repos\Assets - Copy\Assets\ClientApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA6F932A-5193-4317-994E-8EF866FD9674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D8C6814-A075-4457-97CE-1326B6F7EA4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="795" yWindow="1350" windowWidth="14775" windowHeight="11295" xr2:uid="{18E49AEB-C42B-4258-B93E-42E65A904A90}"/>
+    <workbookView minimized="1" xWindow="795" yWindow="1350" windowWidth="14775" windowHeight="11295" xr2:uid="{18E49AEB-C42B-4258-B93E-42E65A904A90}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -3363,6 +3363,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5F7E328-366C-430D-80B7-57A4E09F4F93}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G224"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3399,7 +3400,7 @@
         <v>987</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -3422,7 +3423,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -3445,7 +3446,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -3468,7 +3469,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -3491,7 +3492,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>20</v>
       </c>
@@ -3537,7 +3538,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
@@ -3560,7 +3561,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>32</v>
       </c>
@@ -3583,7 +3584,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>37</v>
       </c>
@@ -3606,7 +3607,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -3629,7 +3630,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>46</v>
       </c>
@@ -3652,7 +3653,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>50</v>
       </c>
@@ -3675,7 +3676,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>55</v>
       </c>
@@ -3698,7 +3699,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>60</v>
       </c>
@@ -3721,7 +3722,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>65</v>
       </c>
@@ -3744,7 +3745,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>70</v>
       </c>
@@ -3767,7 +3768,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>75</v>
       </c>
@@ -3790,7 +3791,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>80</v>
       </c>
@@ -3813,7 +3814,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>85</v>
       </c>
@@ -3836,7 +3837,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>90</v>
       </c>
@@ -3859,7 +3860,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>95</v>
       </c>
@@ -3882,7 +3883,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>100</v>
       </c>
@@ -3905,7 +3906,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>105</v>
       </c>
@@ -3928,7 +3929,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>109</v>
       </c>
@@ -3951,7 +3952,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>113</v>
       </c>
@@ -3974,7 +3975,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>117</v>
       </c>
@@ -3997,7 +3998,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>122</v>
       </c>
@@ -4020,7 +4021,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>127</v>
       </c>
@@ -4043,7 +4044,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>131</v>
       </c>
@@ -4066,7 +4067,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>135</v>
       </c>
@@ -4089,7 +4090,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>139</v>
       </c>
@@ -4112,7 +4113,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>143</v>
       </c>
@@ -4135,7 +4136,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>148</v>
       </c>
@@ -4158,7 +4159,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>153</v>
       </c>
@@ -4181,7 +4182,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>157</v>
       </c>
@@ -4204,7 +4205,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>162</v>
       </c>
@@ -4227,7 +4228,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>166</v>
       </c>
@@ -4273,7 +4274,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>174</v>
       </c>
@@ -4296,7 +4297,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>179</v>
       </c>
@@ -4319,7 +4320,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>183</v>
       </c>
@@ -4342,7 +4343,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>187</v>
       </c>
@@ -4365,7 +4366,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>192</v>
       </c>
@@ -4388,7 +4389,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>195</v>
       </c>
@@ -4411,7 +4412,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>200</v>
       </c>
@@ -4434,7 +4435,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>204</v>
       </c>
@@ -4457,7 +4458,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>208</v>
       </c>
@@ -4480,7 +4481,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>211</v>
       </c>
@@ -4503,7 +4504,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>215</v>
       </c>
@@ -4526,7 +4527,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>220</v>
       </c>
@@ -4549,7 +4550,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>224</v>
       </c>
@@ -4572,7 +4573,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>228</v>
       </c>
@@ -4595,7 +4596,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>231</v>
       </c>
@@ -4618,7 +4619,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>234</v>
       </c>
@@ -4641,7 +4642,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>237</v>
       </c>
@@ -4664,7 +4665,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>240</v>
       </c>
@@ -4687,7 +4688,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>243</v>
       </c>
@@ -4710,7 +4711,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>246</v>
       </c>
@@ -4733,7 +4734,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>249</v>
       </c>
@@ -4756,7 +4757,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>253</v>
       </c>
@@ -4779,7 +4780,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>256</v>
       </c>
@@ -4802,7 +4803,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>260</v>
       </c>
@@ -4825,7 +4826,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>265</v>
       </c>
@@ -4848,7 +4849,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>270</v>
       </c>
@@ -4871,7 +4872,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>275</v>
       </c>
@@ -4894,7 +4895,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>279</v>
       </c>
@@ -4917,7 +4918,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>284</v>
       </c>
@@ -4940,7 +4941,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>289</v>
       </c>
@@ -4963,7 +4964,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>293</v>
       </c>
@@ -4986,7 +4987,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>297</v>
       </c>
@@ -5009,7 +5010,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>302</v>
       </c>
@@ -5032,7 +5033,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>307</v>
       </c>
@@ -5055,7 +5056,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>312</v>
       </c>
@@ -5078,7 +5079,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>317</v>
       </c>
@@ -5101,7 +5102,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>322</v>
       </c>
@@ -5124,7 +5125,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>327</v>
       </c>
@@ -5147,7 +5148,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>332</v>
       </c>
@@ -5170,7 +5171,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>337</v>
       </c>
@@ -5193,7 +5194,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>342</v>
       </c>
@@ -5216,7 +5217,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>346</v>
       </c>
@@ -5239,7 +5240,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>351</v>
       </c>
@@ -5262,7 +5263,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>356</v>
       </c>
@@ -5285,7 +5286,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>361</v>
       </c>
@@ -5308,7 +5309,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>365</v>
       </c>
@@ -5331,7 +5332,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>370</v>
       </c>
@@ -5354,7 +5355,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>374</v>
       </c>
@@ -5377,7 +5378,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>378</v>
       </c>
@@ -5400,7 +5401,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>383</v>
       </c>
@@ -5423,7 +5424,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>388</v>
       </c>
@@ -5446,7 +5447,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>393</v>
       </c>
@@ -5469,7 +5470,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>397</v>
       </c>
@@ -5492,7 +5493,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>402</v>
       </c>
@@ -5515,7 +5516,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>407</v>
       </c>
@@ -5538,7 +5539,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>412</v>
       </c>
@@ -5561,7 +5562,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>416</v>
       </c>
@@ -5584,7 +5585,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>420</v>
       </c>
@@ -5607,7 +5608,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>424</v>
       </c>
@@ -5630,7 +5631,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>428</v>
       </c>
@@ -5653,7 +5654,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>433</v>
       </c>
@@ -5676,7 +5677,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>437</v>
       </c>
@@ -5699,7 +5700,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>442</v>
       </c>
@@ -5722,7 +5723,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>447</v>
       </c>
@@ -5745,7 +5746,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>452</v>
       </c>
@@ -5768,7 +5769,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>456</v>
       </c>
@@ -5791,7 +5792,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>460</v>
       </c>
@@ -5814,7 +5815,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>465</v>
       </c>
@@ -5837,7 +5838,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>469</v>
       </c>
@@ -5860,7 +5861,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>473</v>
       </c>
@@ -5883,7 +5884,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>478</v>
       </c>
@@ -5906,7 +5907,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>483</v>
       </c>
@@ -5929,7 +5930,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>487</v>
       </c>
@@ -5952,7 +5953,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>492</v>
       </c>
@@ -5975,7 +5976,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>497</v>
       </c>
@@ -5998,7 +5999,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>501</v>
       </c>
@@ -6021,7 +6022,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>506</v>
       </c>
@@ -6044,7 +6045,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>511</v>
       </c>
@@ -6067,7 +6068,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>515</v>
       </c>
@@ -6090,7 +6091,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>519</v>
       </c>
@@ -6113,7 +6114,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>524</v>
       </c>
@@ -6136,7 +6137,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>528</v>
       </c>
@@ -6159,7 +6160,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>533</v>
       </c>
@@ -6182,7 +6183,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>537</v>
       </c>
@@ -6205,7 +6206,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>541</v>
       </c>
@@ -6228,7 +6229,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>545</v>
       </c>
@@ -6251,7 +6252,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>550</v>
       </c>
@@ -6274,7 +6275,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>554</v>
       </c>
@@ -6297,7 +6298,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>558</v>
       </c>
@@ -6320,7 +6321,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>562</v>
       </c>
@@ -6343,7 +6344,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>566</v>
       </c>
@@ -6366,7 +6367,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>571</v>
       </c>
@@ -6389,7 +6390,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>575</v>
       </c>
@@ -6412,7 +6413,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>579</v>
       </c>
@@ -6435,7 +6436,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>584</v>
       </c>
@@ -6458,7 +6459,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>589</v>
       </c>
@@ -6481,7 +6482,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>594</v>
       </c>
@@ -6504,7 +6505,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>598</v>
       </c>
@@ -6527,7 +6528,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>603</v>
       </c>
@@ -6550,7 +6551,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>608</v>
       </c>
@@ -6573,7 +6574,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>613</v>
       </c>
@@ -6596,7 +6597,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>617</v>
       </c>
@@ -6619,7 +6620,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>621</v>
       </c>
@@ -6642,7 +6643,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>626</v>
       </c>
@@ -6665,7 +6666,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>630</v>
       </c>
@@ -6688,7 +6689,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>635</v>
       </c>
@@ -6711,7 +6712,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>639</v>
       </c>
@@ -6734,7 +6735,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>643</v>
       </c>
@@ -6757,7 +6758,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>647</v>
       </c>
@@ -6780,7 +6781,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>652</v>
       </c>
@@ -6803,7 +6804,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>656</v>
       </c>
@@ -6849,7 +6850,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>664</v>
       </c>
@@ -6872,7 +6873,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>668</v>
       </c>
@@ -6895,7 +6896,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>673</v>
       </c>
@@ -6918,7 +6919,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>677</v>
       </c>
@@ -6964,7 +6965,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>686</v>
       </c>
@@ -6987,7 +6988,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>691</v>
       </c>
@@ -7010,7 +7011,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>695</v>
       </c>
@@ -7033,7 +7034,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>700</v>
       </c>
@@ -7056,7 +7057,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>705</v>
       </c>
@@ -7079,7 +7080,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>710</v>
       </c>
@@ -7102,7 +7103,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>714</v>
       </c>
@@ -7125,7 +7126,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>719</v>
       </c>
@@ -7148,7 +7149,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>724</v>
       </c>
@@ -7171,7 +7172,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>728</v>
       </c>
@@ -7194,7 +7195,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>732</v>
       </c>
@@ -7217,7 +7218,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>736</v>
       </c>
@@ -7240,7 +7241,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>741</v>
       </c>
@@ -7263,7 +7264,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>745</v>
       </c>
@@ -7286,7 +7287,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>750</v>
       </c>
@@ -7309,7 +7310,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>754</v>
       </c>
@@ -7332,7 +7333,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>759</v>
       </c>
@@ -7355,7 +7356,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>763</v>
       </c>
@@ -7378,7 +7379,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>768</v>
       </c>
@@ -7401,7 +7402,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
         <v>772</v>
       </c>
@@ -7424,7 +7425,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
         <v>776</v>
       </c>
@@ -7447,7 +7448,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
         <v>780</v>
       </c>
@@ -7470,7 +7471,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>784</v>
       </c>
@@ -7493,7 +7494,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
         <v>788</v>
       </c>
@@ -7516,7 +7517,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>792</v>
       </c>
@@ -7539,7 +7540,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>796</v>
       </c>
@@ -7562,7 +7563,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>801</v>
       </c>
@@ -7585,7 +7586,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
         <v>804</v>
       </c>
@@ -7608,7 +7609,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
         <v>808</v>
       </c>
@@ -7631,7 +7632,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
         <v>812</v>
       </c>
@@ -7654,7 +7655,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
         <v>816</v>
       </c>
@@ -7677,7 +7678,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>820</v>
       </c>
@@ -7700,7 +7701,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
         <v>824</v>
       </c>
@@ -7723,7 +7724,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
         <v>829</v>
       </c>
@@ -7746,7 +7747,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>832</v>
       </c>
@@ -7769,7 +7770,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
         <v>835</v>
       </c>
@@ -7792,7 +7793,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
         <v>838</v>
       </c>
@@ -7815,7 +7816,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>841</v>
       </c>
@@ -7838,7 +7839,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>844</v>
       </c>
@@ -7861,7 +7862,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>847</v>
       </c>
@@ -7884,7 +7885,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
         <v>850</v>
       </c>
@@ -7907,7 +7908,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
         <v>853</v>
       </c>
@@ -7930,7 +7931,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>856</v>
       </c>
@@ -7953,7 +7954,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>860</v>
       </c>
@@ -7976,7 +7977,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
         <v>864</v>
       </c>
@@ -7999,7 +8000,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
         <v>868</v>
       </c>
@@ -8022,7 +8023,7 @@
         <v>871</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
         <v>872</v>
       </c>
@@ -8045,7 +8046,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>877</v>
       </c>
@@ -8068,7 +8069,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
         <v>881</v>
       </c>
@@ -8091,7 +8092,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
         <v>884</v>
       </c>
@@ -8114,7 +8115,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>887</v>
       </c>
@@ -8137,7 +8138,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
         <v>891</v>
       </c>
@@ -8160,7 +8161,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
         <v>894</v>
       </c>
@@ -8183,7 +8184,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
         <v>897</v>
       </c>
@@ -8206,7 +8207,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
         <v>900</v>
       </c>
@@ -8229,7 +8230,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
         <v>904</v>
       </c>
@@ -8252,7 +8253,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
         <v>908</v>
       </c>
@@ -8275,7 +8276,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
         <v>913</v>
       </c>
@@ -8298,7 +8299,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
         <v>917</v>
       </c>
@@ -8321,7 +8322,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
         <v>921</v>
       </c>
@@ -8344,7 +8345,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
         <v>925</v>
       </c>
@@ -8367,7 +8368,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
         <v>929</v>
       </c>
@@ -8390,7 +8391,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
         <v>933</v>
       </c>
@@ -8413,7 +8414,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>937</v>
       </c>
@@ -8436,7 +8437,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
         <v>941</v>
       </c>
@@ -8459,7 +8460,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
         <v>946</v>
       </c>
@@ -8482,7 +8483,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
         <v>950</v>
       </c>
@@ -8505,7 +8506,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
         <v>954</v>
       </c>
@@ -8529,7 +8530,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G224" xr:uid="{C5F7E328-366C-430D-80B7-57A4E09F4F93}"/>
+  <autoFilter ref="A1:G224" xr:uid="{C5F7E328-366C-430D-80B7-57A4E09F4F93}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="&quot;محمد علاء&quot; عبد الرحمن محمد دراويش"/>
+        <filter val="علاء احمد ذيب ابو حماد"/>
+        <filter val="علاء عيسى علي عمرو"/>
+        <filter val="محمد علاء عايد محمد عرجان"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>